<commit_message>
Separated function files, added comorbidity
</commit_message>
<xml_diff>
--- a/adhd_adults_diagnosis_SoF.xlsx
+++ b/adhd_adults_diagnosis_SoF.xlsx
@@ -379,12 +379,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>3 studies (Groom, 2016{#325}; Pettersson, 2018{#711}; Kingston, 2013{#5349})</t>
+          <t>5 studies (Groom, 2016{#325}; Lancaster, 2018{#495}; Pettersson, 2018{#711}; Chen, 2021{#5100}; Kingston, 2013{#5349})</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>16(#325) to 18(#5349)</t>
+          <t>14(#495) to 37(#5100)</t>
         </is>
       </c>
     </row>
@@ -396,12 +396,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>10 studies (Groom, 2016{#325}; Pettersson, 2018{#711}; Van Voorhees, 2011{#949}; Kingston, 2013{#5349}; Dvorsky, 2016{#10626}; Robeva, 2004{#10732}; Ma, 2025{#11059}; Wiebe, 2024{#11135}; Zhu, 2026{#13862}; Bijlenga, 2019{#14652})</t>
+          <t>12 studies (Groom, 2016{#325}; Lancaster, 2018{#495}; Pettersson, 2018{#711}; Van Voorhees, 2011{#949}; Kingston, 2013{#5349}; Dvorsky, 2016{#10626}; Robeva, 2004{#10732}; Ma, 2025{#11059}; Wiebe, 2024{#11135}; Zhu, 2026{#13862}; Kautzky, 2020{#14586}; Bijlenga, 2019{#14652})</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>100(#10732) to 43(#949)</t>
+          <t>100(#10732) to 53(#949)</t>
         </is>
       </c>
     </row>
@@ -413,7 +413,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10 studies (Groom, 2016{#325}; Pettersson, 2018{#711}; Van Voorhees, 2011{#949}; Kingston, 2013{#5349}; Dvorsky, 2016{#10626}; Robeva, 2004{#10732}; Ma, 2025{#11059}; Wiebe, 2024{#11135}; Zhu, 2026{#13862}; Bijlenga, 2019{#14652})</t>
+          <t>12 studies (Groom, 2016{#325}; Lancaster, 2018{#495}; Pettersson, 2018{#711}; Van Voorhees, 2011{#949}; Kingston, 2013{#5349}; Dvorsky, 2016{#10626}; Robeva, 2004{#10732}; Ma, 2025{#11059}; Wiebe, 2024{#11135}; Zhu, 2026{#13862}; Kautzky, 2020{#14586}; Bijlenga, 2019{#14652})</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -515,7 +515,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>25 studies (Bakare, 2020{#45}; Bastiaens, 2017{#55}; Dakwar, 2012{#172}; Grogan, 2018{#323}; Houston, 2011{#390}; Kwan, 2024{#490}; Lancaster, 2018{#495}; Liu, 2023{#536}; Luty, 2009{#555}; Marchant, 2015{#571}; McCann, 2004{#603}; Mehringer, 2002{#611}; Palmer, 2023{#685}; Pettersson, 2018{#711}; Reimherr, 2021{#757}; Reyes, 2019{#762}; Singh, 2015{#857}; Solanto, 2004{#870}; van de Glind, 2013{#942}; Young, 2023{#1016}; Kumar, 2011{#4185}; Kingston, 2013{#5349}; Knight, 2025{#11044}; Herman, 2025{#14009}; Kitsune, 2016{#14746})</t>
+          <t>27 studies (Bakare, 2020{#45}; Bastiaens, 2017{#55}; Dakwar, 2012{#172}; Grogan, 2018{#323}; Harrison, 2019{#351}; Kwan, 2024{#490}; Liu, 2023{#536}; Luty, 2009{#555}; Marchant, 2015{#571}; McCann, 2004{#603}; Mehringer, 2002{#611}; Palmer, 2023{#685}; Pettersson, 2018{#711}; Reimherr, 2021{#757}; Reyes, 2019{#762}; Singh, 2015{#857}; Solanto, 2004{#870}; Ustun, 2017{#940}; van de Glind, 2013{#942}; Young, 2023{#1016}; Kumar, 2011{#4185}; Roy-Byrne, 1997{#4485}; Kingston, 2013{#5349}; Knight, 2025{#11044}; Roman, 2025{#11101}; Herman, 2025{#14009}; Kitsune, 2016{#14746})</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -532,12 +532,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>41 studies (Aita, 2018{#16}; Bakare, 2020{#45}; Bastiaens, 2017{#55}; Chiasson, 2012{#141}; Dakwar, 2012{#172}; Dunlop, 2018{#212}; Grogan, 2018{#323}; Harrison, 2019{#351}; Houston, 2011{#390}; Kessler, 2005{#442}; Kwan, 2024{#490}; Lancaster, 2018{#495}; Lewandowski, 2008{#525}; Liu, 2023{#536}; Luty, 2009{#555}; Marchant, 2015{#571}; McCann, 2004{#603}; Mehringer, 2002{#611}; Palmer, 2023{#685}; Pettersson, 2018{#711}; Reimherr, 2021{#757}; Reyes, 2019{#762}; Singh, 2015{#857}; Solanto, 2004{#870}; Ustun, 2017{#940}; van de Glind, 2013{#942}; Van Voorhees, 2011{#949}; Vizgaitis, 2023{#960}; Young, 2023{#1016}; Young, 2016{#1017}; Kumar, 2011{#4185}; Roy-Byrne, 1997{#4485}; Erhardt, 1999{#5176}; Kingston, 2013{#5349}; De Quiros, 2001{#10619}; Dvorsky, 2016{#10626}; Faraone, 2010{#10633}; Skirrow, 2013{#10752}; Knight, 2025{#11044}; Herman, 2025{#14009}; Kitsune, 2016{#14746})</t>
+          <t>41 studies (Aita, 2018{#16}; Bakare, 2020{#45}; Bastiaens, 2017{#55}; Chiasson, 2012{#141}; Dakwar, 2012{#172}; Dunlop, 2018{#212}; Grogan, 2018{#323}; Harrison, 2019{#351}; Houston, 2011{#390}; Kessler, 2005{#442}; Kwan, 2024{#490}; Lewandowski, 2008{#525}; Liu, 2023{#536}; Luty, 2009{#555}; Marchant, 2015{#571}; McCann, 2004{#603}; Mehringer, 2002{#611}; Palmer, 2023{#685}; Pettersson, 2018{#711}; Reimherr, 2021{#757}; Reyes, 2019{#762}; Singh, 2015{#857}; Solanto, 2004{#870}; Ustun, 2017{#940}; van de Glind, 2013{#942}; Van Voorhees, 2011{#949}; Vizgaitis, 2023{#960}; Young, 2023{#1016}; Young, 2016{#1017}; Kumar, 2011{#4185}; Roy-Byrne, 1997{#4485}; Erhardt, 1999{#5176}; Kingston, 2013{#5349}; De Quiros, 2001{#10619}; Dvorsky, 2016{#10626}; Faraone, 2010{#10633}; Skirrow, 2013{#10752}; Knight, 2025{#11044}; Roman, 2025{#11101}; Herman, 2025{#14009}; Kitsune, 2016{#14746})</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>100(#141, 490) to 14(#351)</t>
+          <t>100(#141, 490) to 33(#11044)</t>
         </is>
       </c>
     </row>
@@ -549,7 +549,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>39 studies (Bakare, 2020{#45}; Bastiaens, 2017{#55}; Dakwar, 2012{#172}; Dunlop, 2018{#212}; Grogan, 2018{#323}; Harrison, 2019{#351}; Houston, 2011{#390}; Kessler, 2005{#442}; Kwan, 2024{#490}; Lancaster, 2018{#495}; Lewandowski, 2008{#525}; Liu, 2023{#536}; Luty, 2009{#555}; Marchant, 2015{#571}; McCann, 2004{#603}; Mehringer, 2002{#611}; Palmer, 2023{#685}; Pettersson, 2018{#711}; Reimherr, 2021{#757}; Reyes, 2019{#762}; Singh, 2015{#857}; Solanto, 2004{#870}; Ustun, 2017{#940}; van de Glind, 2013{#942}; Van Voorhees, 2011{#949}; Vizgaitis, 2023{#960}; Young, 2023{#1016}; Young, 2016{#1017}; Kumar, 2011{#4185}; Roy-Byrne, 1997{#4485}; Erhardt, 1999{#5176}; Kingston, 2013{#5349}; De Quiros, 2001{#10619}; Dvorsky, 2016{#10626}; Faraone, 2010{#10633}; Skirrow, 2013{#10752}; Knight, 2025{#11044}; Herman, 2025{#14009}; Kitsune, 2016{#14746})</t>
+          <t>39 studies (Bakare, 2020{#45}; Bastiaens, 2017{#55}; Dakwar, 2012{#172}; Dunlop, 2018{#212}; Grogan, 2018{#323}; Harrison, 2019{#351}; Houston, 2011{#390}; Kessler, 2005{#442}; Kwan, 2024{#490}; Lewandowski, 2008{#525}; Liu, 2023{#536}; Luty, 2009{#555}; Marchant, 2015{#571}; McCann, 2004{#603}; Mehringer, 2002{#611}; Palmer, 2023{#685}; Pettersson, 2018{#711}; Reimherr, 2021{#757}; Reyes, 2019{#762}; Singh, 2015{#857}; Solanto, 2004{#870}; Ustun, 2017{#940}; van de Glind, 2013{#942}; Van Voorhees, 2011{#949}; Vizgaitis, 2023{#960}; Young, 2023{#1016}; Young, 2016{#1017}; Kumar, 2011{#4185}; Roy-Byrne, 1997{#4485}; Erhardt, 1999{#5176}; Kingston, 2013{#5349}; De Quiros, 2001{#10619}; Dvorsky, 2016{#10626}; Faraone, 2010{#10633}; Skirrow, 2013{#10752}; Knight, 2025{#11044}; Roman, 2025{#11101}; Herman, 2025{#14009}; Kitsune, 2016{#14746})</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -787,12 +787,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>9 studies (Abramson, 2023{#5}; Adamou, 2022{#8}; Brunkhorst-Kanaan, 2020{#111}; Groom, 2016{#325}; Pettersson, 2018{#711}; Soederstroem,  2014{#869}; Shepler, 2024{#4544}; Kingston, 2013{#5349}; Nikolas, 2019{#10710})</t>
+          <t>8 studies (Abramson, 2023{#5}; Adamou, 2022{#8}; Groom, 2016{#325}; Pettersson, 2018{#711}; Soederstroem,  2014{#869}; Shepler, 2024{#4544}; Kingston, 2013{#5349}; Nikolas, 2019{#10710})</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>11(#5) to 60(#869)</t>
+          <t>8(#5) to 60(#869)</t>
         </is>
       </c>
     </row>
@@ -804,12 +804,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>22 studies (Abramson, 2023{#5}; Adamou, 2022{#8}; Brunkhorst-Kanaan, 2020{#111}; Cohen, 2007{#152}; Edebol, 2012{#220}; Emser, 2018{#234}; Groom, 2016{#325}; Mostert, 2015{#638}; Nielsen, 2011{#659}; Pettersson, 2018{#711}; Schreiber, 1999{#818}; Soederstroem,  2014{#869}; Wiig, 2012{#987}; Elbaum, 2020{#3913}; Lev,  2022{#4209}; Rogers, 2021{#4474}; Shepler, 2024{#4544}; Kingston, 2013{#5349}; Nikolas, 2019{#10710}; Ma, 2025{#11059}; Bijlenga, 2019{#14652}; Corbett, 1999{#15056})</t>
+          <t>23 studies (Abramson, 2023{#5}; Adamou, 2022{#8}; Cohen, 2007{#152}; Edebol, 2012{#220}; Emser, 2018{#234}; Groom, 2016{#325}; Lovejoy, 1999{#544}; Mostert, 2015{#638}; Nielsen, 2011{#659}; Pettersson, 2018{#711}; Schreiber, 1999{#818}; Soederstroem,  2014{#869}; Wiig, 2012{#987}; Elbaum, 2020{#3913}; Katz, 1998{#4144}; Lev,  2022{#4209}; Rogers, 2021{#4474}; Shepler, 2024{#4544}; Kingston, 2013{#5349}; Nikolas, 2019{#10710}; Ma, 2025{#11059}; Bijlenga, 2019{#14652}; Corbett, 1999{#15056})</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>93(#659) to 30(#5349)</t>
+          <t>97(#4144) to 39(#5349)</t>
         </is>
       </c>
     </row>
@@ -821,12 +821,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>21 studies (Abramson, 2023{#5}; Adamou, 2022{#8}; Brunkhorst-Kanaan, 2020{#111}; Cohen, 2007{#152}; Edebol, 2012{#220}; Emser, 2018{#234}; Groom, 2016{#325}; Mostert, 2015{#638}; Nielsen, 2011{#659}; Pettersson, 2018{#711}; Schreiber, 1999{#818}; Soederstroem,  2014{#869}; Elbaum, 2020{#3913}; Lev,  2022{#4209}; Rogers, 2021{#4474}; Shepler, 2024{#4544}; Kingston, 2013{#5349}; Nikolas, 2019{#10710}; Ma, 2025{#11059}; Bijlenga, 2019{#14652}; Corbett, 1999{#15056})</t>
+          <t>22 studies (Abramson, 2023{#5}; Adamou, 2022{#8}; Cohen, 2007{#152}; Edebol, 2012{#220}; Emser, 2018{#234}; Groom, 2016{#325}; Lovejoy, 1999{#544}; Mostert, 2015{#638}; Nielsen, 2011{#659}; Pettersson, 2018{#711}; Schreiber, 1999{#818}; Soederstroem,  2014{#869}; Elbaum, 2020{#3913}; Katz, 1998{#4144}; Lev,  2022{#4209}; Rogers, 2021{#4474}; Shepler, 2024{#4544}; Kingston, 2013{#5349}; Nikolas, 2019{#10710}; Ma, 2025{#11059}; Bijlenga, 2019{#14652}; Corbett, 1999{#15056})</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>100(#659) to 40(#869)</t>
+          <t>100(#659) to 40(#869, 4144)</t>
         </is>
       </c>
     </row>
@@ -923,12 +923,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>3 studies (Amen, 2021{#28}; Schneider, 2014{#812}; Solouki, 2025{#13916})</t>
+          <t>2 studies (Schneider, 2014{#812}; Solouki, 2025{#13916})</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>3(#28, 13916) to 24(#812)</t>
+          <t>3(#13916) to 24(#812)</t>
         </is>
       </c>
     </row>
@@ -940,7 +940,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>11 studies (Amen, 2021{#28}; Chaim-Avancini, 2017{#134}; Schneider, 2014{#812}; Wang, 2013{#970}; Yao, 2018{#1011}; Hong, 2024{#11027}; Lim, 2025{#11051}; Ma, 2025{#11059}; Zhu, 2026{#13862}; Solouki, 2025{#13916}; Kautzky, 2020{#14586})</t>
+          <t>12 studies (Amen, 2021{#28}; Chaim-Avancini, 2017{#134}; Schneider, 2014{#812}; Wang, 2013{#970}; Yao, 2018{#1011}; Amen, 2008{#10932}; Hong, 2024{#11027}; Lim, 2025{#11051}; Ma, 2025{#11059}; Zhu, 2026{#13862}; Solouki, 2025{#13916}; Kautzky, 2020{#14586})</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -957,12 +957,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>11 studies (Amen, 2021{#28}; Chaim-Avancini, 2017{#134}; Schneider, 2014{#812}; Wang, 2013{#970}; Yao, 2018{#1011}; Hong, 2024{#11027}; Lim, 2025{#11051}; Ma, 2025{#11059}; Zhu, 2026{#13862}; Solouki, 2025{#13916}; Kautzky, 2020{#14586})</t>
+          <t>12 studies (Amen, 2021{#28}; Chaim-Avancini, 2017{#134}; Schneider, 2014{#812}; Wang, 2013{#970}; Yao, 2018{#1011}; Amen, 2008{#10932}; Hong, 2024{#11027}; Lim, 2025{#11051}; Ma, 2025{#11059}; Zhu, 2026{#13862}; Solouki, 2025{#13916}; Kautzky, 2020{#14586})</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>97(#28, 13916) to 65(#1011)</t>
+          <t>100(#28) to 65(#1011)</t>
         </is>
       </c>
     </row>
@@ -1081,7 +1081,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>100(#436) to 67(#722)</t>
+          <t>100(#436) to 61(#448)</t>
         </is>
       </c>
     </row>
@@ -1098,7 +1098,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>96(#14166) to 37(#448)</t>
+          <t>100(#436) to 48(#448)</t>
         </is>
       </c>
     </row>
@@ -1212,7 +1212,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>7 studies (Grünblatt, 2012{#327}; Jimenez, 2021{#417}; Andrikopoulos, 2024{#5003}; Udal, 2024{#5685}; Ma, 2025{#11059}; von Polier, 2025{#11129}; Zhu, 2026{#13862})</t>
+          <t>8 studies (Grünblatt, 2012{#327}; Jimenez, 2021{#417}; Andrikopoulos, 2024{#5003}; Udal, 2024{#5685}; Ma, 2025{#11059}; von Polier, 2025{#11129}; Zhu, 2026{#13862}; Kautzky, 2020{#14586})</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -1229,7 +1229,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>7 studies (Grünblatt, 2012{#327}; Jimenez, 2021{#417}; Andrikopoulos, 2024{#5003}; Udal, 2024{#5685}; Ma, 2025{#11059}; von Polier, 2025{#11129}; Zhu, 2026{#13862})</t>
+          <t>8 studies (Grünblatt, 2012{#327}; Jimenez, 2021{#417}; Andrikopoulos, 2024{#5003}; Udal, 2024{#5685}; Ma, 2025{#11059}; von Polier, 2025{#11129}; Zhu, 2026{#13862}; Kautzky, 2020{#14586})</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -1744,7 +1744,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>5(#10849) to 22(#11099)</t>
+          <t>5(#10849) to 46(#5)</t>
         </is>
       </c>
     </row>
@@ -1756,7 +1756,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>23 studies (Abramson, 2023{#5}; Aita, 2018{#16}; Becke, 2023{#58}; Berger, 2021{#68}; Courrege, 2019{#164}; Harrison, 2019{#351}; Musso, 2016{#646}; Potts, 2022{#733}; Quinn, 2003{#745}; Ramachandran, 2019{#750}; Robinson, 2023{#777}; Smith, 2017{#863}; Sollman, 2010{#872}; Spenceley, 2022{#883}; Young, 2011{#1015}; Harrison, 2020{#4042}; Morey, 2019{#4321}; Williamson, 2014{#4702}; Fuermaier, 2016{#5208}; Suhr, 2011{#10849}; Fuermaier, 2024{#11004}; Robinson, 2025{#11099}; Robinson, 2023{#14273})</t>
+          <t>23 studies (Abramson, 2023{#5}; Aita, 2018{#16}; Becke, 2023{#58}; Berger, 2021{#68}; Courrege, 2019{#164}; Harrison, 2019{#351}; Musso, 2016{#646}; Potts, 2022{#733}; Quinn, 2003{#745}; Ramachandran, 2019{#750}; Robinson, 2023{#777}; Smith, 2017{#863}; Sollman, 2010{#872}; Spenceley, 2022{#883}; Young, 2011{#1015}; Harrison, 2020{#4042}; Morey, 2019{#4321}; Williamson, 2014{#4702}; Fuermaier, 2016{#5208}; Suhr, 2011{#10849}; Fuermaier, 2024{#11011}; Robinson, 2025{#11099}; Robinson, 2023{#14273})</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -1773,12 +1773,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>21 studies (Abramson, 2023{#5}; Becke, 2023{#58}; Berger, 2021{#68}; Courrege, 2019{#164}; Harrison, 2019{#351}; Musso, 2016{#646}; Potts, 2022{#733}; Quinn, 2003{#745}; Ramachandran, 2019{#750}; Robinson, 2023{#777}; Smith, 2017{#863}; Sollman, 2010{#872}; Spenceley, 2022{#883}; Young, 2011{#1015}; Harrison, 2020{#4042}; Morey, 2019{#4321}; Fuermaier, 2016{#5208}; Suhr, 2011{#10849}; Fuermaier, 2024{#11004}; Robinson, 2025{#11099}; Robinson, 2023{#14273})</t>
+          <t>21 studies (Abramson, 2023{#5}; Becke, 2023{#58}; Berger, 2021{#68}; Courrege, 2019{#164}; Harrison, 2019{#351}; Musso, 2016{#646}; Potts, 2022{#733}; Quinn, 2003{#745}; Ramachandran, 2019{#750}; Robinson, 2023{#777}; Smith, 2017{#863}; Sollman, 2010{#872}; Spenceley, 2022{#883}; Young, 2011{#1015}; Harrison, 2020{#4042}; Morey, 2019{#4321}; Fuermaier, 2016{#5208}; Suhr, 2011{#10849}; Fuermaier, 2024{#11011}; Robinson, 2025{#11099}; Robinson, 2023{#14273})</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>98(#646) to 78(#11099)</t>
+          <t>98(#646) to 54(#5)</t>
         </is>
       </c>
     </row>

</xml_diff>